<commit_message>
Cleaned and new biodiv source data changed
</commit_message>
<xml_diff>
--- a/Raw_Data/v6b_CLempN_exc_allecosys.xlsx
+++ b/Raw_Data/v6b_CLempN_exc_allecosys.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StefanÅström\C_Verktyg\Python\ALL_PYTHON\CBA_GOT_PROT\CBA_GBG_PROT\Raw_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anthesisllc-my.sharepoint.com/personal/lovisa_areback_anthesisgroup_com/Documents/Dokument/GitHub/2026_v6b2_Goth_Prot_CBA/Raw_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278B948F-6F86-4A06-9695-60754D0CCEC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{278B948F-6F86-4A06-9695-60754D0CCEC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54B3396F-F562-422B-BCEE-E7F494F47F6F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A5EB80D3-E071-4672-B953-6567AA6F42B9}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="11143" windowHeight="13080" firstSheet="3" activeTab="7" xr2:uid="{A5EB80D3-E071-4672-B953-6567AA6F42B9}"/>
   </bookViews>
   <sheets>
     <sheet name="clempn_exc_allecosys (19)" sheetId="9" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="clempn_exc_allecosys (20)" sheetId="4" r:id="rId6"/>
     <sheet name="clempn_exc_allecosys (22)" sheetId="3" r:id="rId7"/>
     <sheet name="clempn_exc_allecosys (23)" sheetId="2" r:id="rId8"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -644,39 +643,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265D84C1-98C0-4F57-AA76-BF100C890B97}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -714,7 +713,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -758,7 +757,7 @@
         <v>58.292999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -802,7 +801,7 @@
         <v>217.6568</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -846,7 +845,7 @@
         <v>33.368200000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -890,7 +889,7 @@
         <v>29.666499999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -934,7 +933,7 @@
         <v>65.975899999999996</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -978,7 +977,7 @@
         <v>25.476500000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1022,7 +1021,7 @@
         <v>78.169399999999996</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1066,7 +1065,7 @@
         <v>5.6599999999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1110,7 +1109,7 @@
         <v>5.5999999999999999E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1154,7 +1153,7 @@
         <v>37.389000000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -1198,7 +1197,7 @@
         <v>131.56020000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>36.907299999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -1286,7 +1285,7 @@
         <v>146.21629999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1330,7 +1329,7 @@
         <v>78.2654</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1374,7 +1373,7 @@
         <v>139.0487</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1418,7 +1417,7 @@
         <v>0.53790000000000004</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1462,7 +1461,7 @@
         <v>9.5762999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -1506,7 +1505,7 @@
         <v>16.884</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1550,7 +1549,7 @@
         <v>156.0694</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1594,7 +1593,7 @@
         <v>848.15899999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1638,7 +1637,7 @@
         <v>47.424300000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>39.916499999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -1726,7 +1725,7 @@
         <v>57.953600000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -1770,7 +1769,7 @@
         <v>36.993600000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -1814,7 +1813,7 @@
         <v>107.1159</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1858,7 +1857,7 @@
         <v>105.97110000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1902,7 +1901,7 @@
         <v>0.1913</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -1943,7 +1942,7 @@
         <v>74.946799999999996</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -1987,7 +1986,7 @@
         <v>68.000200000000007</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -2031,7 +2030,7 @@
         <v>261.21429999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -2075,7 +2074,7 @@
         <v>155.45179999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -2119,7 +2118,7 @@
         <v>108.227</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -2163,7 +2162,7 @@
         <v>13.386900000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -2207,7 +2206,7 @@
         <v>71.807299999999998</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -2251,7 +2250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -2295,7 +2294,7 @@
         <v>27.0594</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -2339,7 +2338,7 @@
         <v>12.5055</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -2383,7 +2382,7 @@
         <v>77.989099999999993</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -2427,7 +2426,7 @@
         <v>8.9695999999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -2471,7 +2470,7 @@
         <v>1.0039</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -2515,7 +2514,7 @@
         <v>1.8233999999999999</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -2559,7 +2558,7 @@
         <v>26.641500000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -2603,7 +2602,7 @@
         <v>102.5908</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -2647,7 +2646,7 @@
         <v>122.867</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -2691,7 +2690,7 @@
         <v>42.824100000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -2735,7 +2734,7 @@
         <v>16.943000000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -2776,7 +2775,7 @@
         <v>23.276199999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -2825,39 +2824,39 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D74B54D-A4B0-40A7-B4D7-6F646045B694}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -2895,7 +2894,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -2939,7 +2938,7 @@
         <v>92.531099999999995</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -2983,7 +2982,7 @@
         <v>296.66570000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -3027,7 +3026,7 @@
         <v>58.658299999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -3071,7 +3070,7 @@
         <v>48.991599999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -3115,7 +3114,7 @@
         <v>112.1884</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -3159,7 +3158,7 @@
         <v>35.5366</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -3203,7 +3202,7 @@
         <v>111.0797</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -3247,7 +3246,7 @@
         <v>0.1089</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -3291,7 +3290,7 @@
         <v>1.5100000000000001E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -3335,7 +3334,7 @@
         <v>53.637500000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -3379,7 +3378,7 @@
         <v>165.5445</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -3423,7 +3422,7 @@
         <v>67.415199999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -3467,7 +3466,7 @@
         <v>198.10290000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -3511,7 +3510,7 @@
         <v>89.396100000000004</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -3555,7 +3554,7 @@
         <v>185.35749999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -3599,7 +3598,7 @@
         <v>1.1700999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -3643,7 +3642,7 @@
         <v>16.7761</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -3687,7 +3686,7 @@
         <v>62.228499999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -3731,7 +3730,7 @@
         <v>189.38210000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -3775,7 +3774,7 @@
         <v>926.75130000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -3819,7 +3818,7 @@
         <v>70.857200000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -3863,7 +3862,7 @@
         <v>53.168599999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -3907,7 +3906,7 @@
         <v>76.779899999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -3951,7 +3950,7 @@
         <v>53.704999999999998</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -3995,7 +3994,7 @@
         <v>152.85069999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -4039,7 +4038,7 @@
         <v>149.49199999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -4083,7 +4082,7 @@
         <v>0.32600000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -4124,7 +4123,7 @@
         <v>99.572100000000006</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -4168,7 +4167,7 @@
         <v>118.7353</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -4212,7 +4211,7 @@
         <v>399.4316</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -4256,7 +4255,7 @@
         <v>272.27960000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -4300,7 +4299,7 @@
         <v>165.61340000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -4344,7 +4343,7 @@
         <v>22.1798</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -4388,7 +4387,7 @@
         <v>151.18350000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -4432,7 +4431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -4476,7 +4475,7 @@
         <v>61.883299999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -4520,7 +4519,7 @@
         <v>27.297499999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -4564,7 +4563,7 @@
         <v>136.15870000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -4608,7 +4607,7 @@
         <v>14.4513</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -4652,7 +4651,7 @@
         <v>2.0282</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -4696,7 +4695,7 @@
         <v>5.0273000000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -4740,7 +4739,7 @@
         <v>136.01499999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -4784,7 +4783,7 @@
         <v>127.78530000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -4828,7 +4827,7 @@
         <v>229.3081</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -4872,7 +4871,7 @@
         <v>123.82340000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -4916,7 +4915,7 @@
         <v>26.872800000000002</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -4957,7 +4956,7 @@
         <v>43.463799999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -5006,39 +5005,39 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1FED9B3-3B3C-4CF4-995F-521940700A34}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -5076,7 +5075,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -5120,7 +5119,7 @@
         <v>59.048000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -5164,7 +5163,7 @@
         <v>224.4616</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -5208,7 +5207,7 @@
         <v>43.093299999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -5252,7 +5251,7 @@
         <v>32.0291</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -5296,7 +5295,7 @@
         <v>85.1678</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -5340,7 +5339,7 @@
         <v>25.544799999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -5384,7 +5383,7 @@
         <v>78.637100000000004</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -5428,7 +5427,7 @@
         <v>5.0299999999999997E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -5472,7 +5471,7 @@
         <v>4.7999999999999996E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -5516,7 +5515,7 @@
         <v>43.096499999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -5560,7 +5559,7 @@
         <v>133.166</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -5604,7 +5603,7 @@
         <v>46.527500000000003</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -5648,7 +5647,7 @@
         <v>147.3125</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -5692,7 +5691,7 @@
         <v>83.156300000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -5736,7 +5735,7 @@
         <v>141.68940000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -5780,7 +5779,7 @@
         <v>0.50060000000000004</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -5824,7 +5823,7 @@
         <v>8.2164000000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -5868,7 +5867,7 @@
         <v>19.8599</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -5912,7 +5911,7 @@
         <v>158.4982</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -5956,7 +5955,7 @@
         <v>853.15219999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -6000,7 +5999,7 @@
         <v>46.2759</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -6044,7 +6043,7 @@
         <v>43.310099999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -6088,7 +6087,7 @@
         <v>59.243600000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -6132,7 +6131,7 @@
         <v>37.126199999999997</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -6176,7 +6175,7 @@
         <v>109.45650000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -6220,7 +6219,7 @@
         <v>127.12179999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -6264,7 +6263,7 @@
         <v>0.1885</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -6305,7 +6304,7 @@
         <v>80.370400000000004</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -6349,7 +6348,7 @@
         <v>95.087900000000005</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -6393,7 +6392,7 @@
         <v>295.02080000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -6437,7 +6436,7 @@
         <v>190.4391</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -6481,7 +6480,7 @@
         <v>72.314700000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -6525,7 +6524,7 @@
         <v>14.284000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -6569,7 +6568,7 @@
         <v>91.523499999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -6613,7 +6612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -6657,7 +6656,7 @@
         <v>43.3294</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -6701,7 +6700,7 @@
         <v>16.380400000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -6745,7 +6744,7 @@
         <v>78.810199999999995</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -6789,7 +6788,7 @@
         <v>10.9757</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -6833,7 +6832,7 @@
         <v>1.2414000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -6877,7 +6876,7 @@
         <v>2.0312000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -6921,7 +6920,7 @@
         <v>27.451799999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -6965,7 +6964,7 @@
         <v>104.5455</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -7009,7 +7008,7 @@
         <v>144.2704</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -7053,7 +7052,7 @@
         <v>37.838900000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -7097,7 +7096,7 @@
         <v>17.494499999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -7138,7 +7137,7 @@
         <v>26.682500000000001</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -7187,39 +7186,39 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77835A7E-645E-4A6A-9D4F-4424B4E2A0AE}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -7257,7 +7256,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -7301,7 +7300,7 @@
         <v>30.097000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -7345,7 +7344,7 @@
         <v>154.34780000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -7389,7 +7388,7 @@
         <v>23.853899999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -7433,7 +7432,7 @@
         <v>20.439399999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -7477,7 +7476,7 @@
         <v>51.232399999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -7521,7 +7520,7 @@
         <v>18.6143</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -7565,7 +7564,7 @@
         <v>59.415799999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -7609,7 +7608,7 @@
         <v>2.8999999999999998E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -7653,7 +7652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -7697,7 +7696,7 @@
         <v>27.352799999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7741,7 +7740,7 @@
         <v>83.2102</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -7785,7 +7784,7 @@
         <v>27.302800000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -7829,7 +7828,7 @@
         <v>104.54689999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -7873,7 +7872,7 @@
         <v>49.990299999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -7917,7 +7916,7 @@
         <v>119.4988</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -7961,7 +7960,7 @@
         <v>0.156</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -8005,7 +8004,7 @@
         <v>1.4982</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -8049,7 +8048,7 @@
         <v>8.4265000000000008</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -8093,7 +8092,7 @@
         <v>145.36770000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -8137,7 +8136,7 @@
         <v>767.76580000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -8181,7 +8180,7 @@
         <v>21.5105</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -8225,7 +8224,7 @@
         <v>24.530100000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -8269,7 +8268,7 @@
         <v>40.413800000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -8313,7 +8312,7 @@
         <v>23.87</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -8357,7 +8356,7 @@
         <v>76.5471</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -8401,7 +8400,7 @@
         <v>83.692499999999995</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -8445,7 +8444,7 @@
         <v>7.0199999999999999E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -8486,7 +8485,7 @@
         <v>56.703499999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -8530,7 +8529,7 @@
         <v>58.6464</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -8574,7 +8573,7 @@
         <v>244.01009999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -8618,7 +8617,7 @@
         <v>125.289</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -8662,7 +8661,7 @@
         <v>11.6533</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -8706,7 +8705,7 @@
         <v>9.6951999999999998</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -8750,7 +8749,7 @@
         <v>57.947299999999998</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -8794,7 +8793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -8838,7 +8837,7 @@
         <v>17.4483</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -8882,7 +8881,7 @@
         <v>7.5362</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -8926,7 +8925,7 @@
         <v>20.098400000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -8970,7 +8969,7 @@
         <v>7.5289999999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -9014,7 +9013,7 @@
         <v>0.3957</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -9058,7 +9057,7 @@
         <v>0.76280000000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -9102,7 +9101,7 @@
         <v>18.334599999999998</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -9146,7 +9145,7 @@
         <v>86.155000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -9190,7 +9189,7 @@
         <v>111.9983</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -9234,7 +9233,7 @@
         <v>4.7605000000000004</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -9278,7 +9277,7 @@
         <v>9.5028000000000006</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -9319,7 +9318,7 @@
         <v>18.9877</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -9368,39 +9367,39 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F26C3D-24D7-42D5-81D1-6C49AA36E7D0}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -9438,7 +9437,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -9482,7 +9481,7 @@
         <v>52.495699999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -9526,7 +9525,7 @@
         <v>225.19659999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -9570,7 +9569,7 @@
         <v>33.470599999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -9614,7 +9613,7 @@
         <v>31.2087</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -9658,7 +9657,7 @@
         <v>74.423599999999993</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -9702,7 +9701,7 @@
         <v>25.240600000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -9746,7 +9745,7 @@
         <v>78.477099999999993</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -9790,7 +9789,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -9834,7 +9833,7 @@
         <v>4.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -9878,7 +9877,7 @@
         <v>42.465499999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -9922,7 +9921,7 @@
         <v>132.0421</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -9966,7 +9965,7 @@
         <v>38.255099999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -10010,7 +10009,7 @@
         <v>145.7311</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -10054,7 +10053,7 @@
         <v>83.096199999999996</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -10098,7 +10097,7 @@
         <v>140.80160000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -10142,7 +10141,7 @@
         <v>0.48570000000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -10186,7 +10185,7 @@
         <v>7.6555999999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -10230,7 +10229,7 @@
         <v>18.576599999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -10274,7 +10273,7 @@
         <v>158.20679999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -10318,7 +10317,7 @@
         <v>852.91449999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -10362,7 +10361,7 @@
         <v>46.011499999999998</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -10406,7 +10405,7 @@
         <v>42.348100000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -10450,7 +10449,7 @@
         <v>57.715899999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -10494,7 +10493,7 @@
         <v>36.613700000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -10538,7 +10537,7 @@
         <v>106.5951</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -10582,7 +10581,7 @@
         <v>117.10299999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -10626,7 +10625,7 @@
         <v>0.18720000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -10667,7 +10666,7 @@
         <v>77.732900000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -10711,7 +10710,7 @@
         <v>90.366200000000006</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -10755,7 +10754,7 @@
         <v>269.48590000000002</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -10799,7 +10798,7 @@
         <v>174.50790000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -10843,7 +10842,7 @@
         <v>66.126400000000004</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -10887,7 +10886,7 @@
         <v>13.9551</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -10931,7 +10930,7 @@
         <v>76.414699999999996</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -10975,7 +10974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -11019,7 +11018,7 @@
         <v>29.009</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -11063,7 +11062,7 @@
         <v>13.262499999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -11107,7 +11106,7 @@
         <v>75.938500000000005</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -11151,7 +11150,7 @@
         <v>10.4361</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -11195,7 +11194,7 @@
         <v>1.2352000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -11239,7 +11238,7 @@
         <v>1.8036000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -11283,7 +11282,7 @@
         <v>26.757000000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -11327,7 +11326,7 @@
         <v>99.471199999999996</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -11371,7 +11370,7 @@
         <v>128.101</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -11415,7 +11414,7 @@
         <v>35.9681</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -11459,7 +11458,7 @@
         <v>17.463899999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -11500,7 +11499,7 @@
         <v>23.9727</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -11549,39 +11548,39 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60153BCE-779C-4520-BC60-E8FFF77E2481}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -11619,7 +11618,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -11663,7 +11662,7 @@
         <v>45.896700000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -11707,7 +11706,7 @@
         <v>203.10489999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -11751,7 +11750,7 @@
         <v>26.663799999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -11795,7 +11794,7 @@
         <v>22.257200000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -11839,7 +11838,7 @@
         <v>52.114699999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -11883,7 +11882,7 @@
         <v>22.893599999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -11927,7 +11926,7 @@
         <v>73.683599999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -11971,7 +11970,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -12015,7 +12014,7 @@
         <v>1.9E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -12059,7 +12058,7 @@
         <v>29.910699999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -12103,7 +12102,7 @@
         <v>120.9482</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -12147,7 +12146,7 @@
         <v>29.174800000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -12191,7 +12190,7 @@
         <v>120.7915</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -12235,7 +12234,7 @@
         <v>74.683199999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -12279,7 +12278,7 @@
         <v>123.7313</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -12323,7 +12322,7 @@
         <v>0.38840000000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -12367,7 +12366,7 @@
         <v>4.9322999999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -12411,7 +12410,7 @@
         <v>11.5619</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -12455,7 +12454,7 @@
         <v>151.1704</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -12499,7 +12498,7 @@
         <v>831.05650000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -12543,7 +12542,7 @@
         <v>33.162300000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -12587,7 +12586,7 @@
         <v>27.034199999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -12631,7 +12630,7 @@
         <v>45.471499999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -12675,7 +12674,7 @@
         <v>28.691800000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -12719,7 +12718,7 @@
         <v>87.572000000000003</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -12763,7 +12762,7 @@
         <v>84.324200000000005</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -12807,7 +12806,7 @@
         <v>0.14940000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -12848,7 +12847,7 @@
         <v>65.157300000000006</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -12892,7 +12891,7 @@
         <v>60.078000000000003</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -12936,7 +12935,7 @@
         <v>245.42609999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -12980,7 +12979,7 @@
         <v>128.19200000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -13024,7 +13023,7 @@
         <v>51.687100000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -13068,7 +13067,7 @@
         <v>10.473800000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -13112,7 +13111,7 @@
         <v>59.679699999999997</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -13156,7 +13155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -13200,7 +13199,7 @@
         <v>19.673200000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -13244,7 +13243,7 @@
         <v>8.6417999999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -13288,7 +13287,7 @@
         <v>37.168900000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -13332,7 +13331,7 @@
         <v>7.8304</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -13376,7 +13375,7 @@
         <v>1.0038</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -13420,7 +13419,7 @@
         <v>1.0706</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -13464,7 +13463,7 @@
         <v>21.0669</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -13508,7 +13507,7 @@
         <v>93.118099999999998</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -13552,7 +13551,7 @@
         <v>113.6271</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -13596,7 +13595,7 @@
         <v>20.538699999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -13640,7 +13639,7 @@
         <v>15.934100000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -13681,7 +13680,7 @@
         <v>20.282399999999999</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -13730,39 +13729,39 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9381F60D-B2FA-4766-AD2E-4224BFDDA191}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -13800,7 +13799,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -13844,7 +13843,7 @@
         <v>47.342199999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -13888,7 +13887,7 @@
         <v>222.20840000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -13932,7 +13931,7 @@
         <v>29.9588</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -13976,7 +13975,7 @@
         <v>29.128799999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -14020,7 +14019,7 @@
         <v>65.4054</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -14064,7 +14063,7 @@
         <v>23.806999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -14108,7 +14107,7 @@
         <v>75.877700000000004</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -14152,7 +14151,7 @@
         <v>3.5299999999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -14196,7 +14195,7 @@
         <v>2.8E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -14240,7 +14239,7 @@
         <v>41.255299999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -14284,7 +14283,7 @@
         <v>124.08920000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -14328,7 +14327,7 @@
         <v>33.222299999999997</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -14372,7 +14371,7 @@
         <v>137.88720000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -14416,7 +14415,7 @@
         <v>82.883499999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -14460,7 +14459,7 @@
         <v>137.7064</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -14504,7 +14503,7 @@
         <v>0.4083</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -14548,7 +14547,7 @@
         <v>5.0871000000000004</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -14592,7 +14591,7 @@
         <v>16.994199999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -14636,7 +14635,7 @@
         <v>156.56909999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -14680,7 +14679,7 @@
         <v>844.26220000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -14724,7 +14723,7 @@
         <v>34.286900000000003</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -14768,7 +14767,7 @@
         <v>40.491900000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -14812,7 +14811,7 @@
         <v>50.087299999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -14856,7 +14855,7 @@
         <v>31.609500000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -14900,7 +14899,7 @@
         <v>102.0224</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -14944,7 +14943,7 @@
         <v>110.8506</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -14988,7 +14987,7 @@
         <v>0.15840000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -15029,7 +15028,7 @@
         <v>73.989800000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -15073,7 +15072,7 @@
         <v>75.042199999999994</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -15117,7 +15116,7 @@
         <v>259.31369999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -15161,7 +15160,7 @@
         <v>158.41239999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -15205,7 +15204,7 @@
         <v>57.6723</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -15249,7 +15248,7 @@
         <v>13.268800000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -15293,7 +15292,7 @@
         <v>68.335700000000003</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -15337,7 +15336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -15381,7 +15380,7 @@
         <v>24.713200000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -15425,7 +15424,7 @@
         <v>10.8073</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -15469,7 +15468,7 @@
         <v>49.7485</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -15513,7 +15512,7 @@
         <v>9.4187999999999992</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -15557,7 +15556,7 @@
         <v>1.0664</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -15601,7 +15600,7 @@
         <v>1.5254000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -15645,7 +15644,7 @@
         <v>25.392600000000002</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -15689,7 +15688,7 @@
         <v>96.781300000000002</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -15733,7 +15732,7 @@
         <v>119.5402</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -15777,7 +15776,7 @@
         <v>27.098199999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -15821,7 +15820,7 @@
         <v>17.385300000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -15862,7 +15861,7 @@
         <v>22.163</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -15911,39 +15910,39 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3304473-6B07-46B6-8380-2AE2F48FDC00}">
   <dimension ref="A2:N57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="C9" t="s">
         <v>61</v>
       </c>
@@ -15981,7 +15980,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -16025,7 +16024,7 @@
         <v>35.985300000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -16069,7 +16068,7 @@
         <v>204.47839999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -16113,7 +16112,7 @@
         <v>25.641400000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -16157,7 +16156,7 @@
         <v>22.575099999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -16201,7 +16200,7 @@
         <v>52.978000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -16245,7 +16244,7 @@
         <v>20.660799999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -16289,7 +16288,7 @@
         <v>70.482100000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -16333,7 +16332,7 @@
         <v>2.0899999999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -16377,7 +16376,7 @@
         <v>1.2999999999999999E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -16421,7 +16420,7 @@
         <v>32.661999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -16465,7 +16464,7 @@
         <v>97.901600000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -16509,7 +16508,7 @@
         <v>28.854199999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -16553,7 +16552,7 @@
         <v>112.315</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -16597,7 +16596,7 @@
         <v>80.441299999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -16641,7 +16640,7 @@
         <v>123.614</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -16685,7 +16684,7 @@
         <v>0.30080000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -16729,7 +16728,7 @@
         <v>3.0949</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -16773,7 +16772,7 @@
         <v>10.434100000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -16817,7 +16816,7 @@
         <v>151.42060000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -16861,7 +16860,7 @@
         <v>811.8347</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -16905,7 +16904,7 @@
         <v>28.3931</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -16949,7 +16948,7 @@
         <v>28.8063</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -16993,7 +16992,7 @@
         <v>43.960299999999997</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -17037,7 +17036,7 @@
         <v>26.6921</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -17081,7 +17080,7 @@
         <v>85.181700000000006</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -17125,7 +17124,7 @@
         <v>85.137900000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -17169,7 +17168,7 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -17210,7 +17209,7 @@
         <v>62.580300000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -17254,7 +17253,7 @@
         <v>60.6554</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -17298,7 +17297,7 @@
         <v>249.821</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -17342,7 +17341,7 @@
         <v>144.45689999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -17386,7 +17385,7 @@
         <v>36.939399999999999</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -17430,7 +17429,7 @@
         <v>10.8179</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -17474,7 +17473,7 @@
         <v>62.569800000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>3</v>
       </c>
@@ -17518,7 +17517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -17562,7 +17561,7 @@
         <v>18.971900000000002</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -17606,7 +17605,7 @@
         <v>8.2484000000000002</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -17650,7 +17649,7 @@
         <v>30.971900000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -17694,7 +17693,7 @@
         <v>7.8834</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -17738,7 +17737,7 @@
         <v>0.91059999999999997</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -17782,7 +17781,7 @@
         <v>1.1735</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -17826,7 +17825,7 @@
         <v>20.1099</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -17870,7 +17869,7 @@
         <v>91.0886</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -17914,7 +17913,7 @@
         <v>113.822</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -17958,7 +17957,7 @@
         <v>13.372400000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -18002,7 +18001,7 @@
         <v>16.437200000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>1</v>
       </c>
@@ -18043,7 +18042,7 @@
         <v>20.4681</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -18087,13 +18086,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FDEF07-F609-49FE-91B2-5E291F981283}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>